<commit_message>
Stage 8 review fixes: C-019
</commit_message>
<xml_diff>
--- a/output/archive/MerrivossData/Client_Work/OB11/MV-2020-088/MV-2020-088_AssayWorksheet_042920_v03.xlsx
+++ b/output/archive/MerrivossData/Client_Work/OB11/MV-2020-088/MV-2020-088_AssayWorksheet_042920_v03.xlsx
@@ -166,7 +166,7 @@
   <commentList>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>CYP2C9 is the most flagged isoform this round; the lipophilic cap variants account for most of the CYP3A4 hits.</t>
+        <t>CYP2C9 and CYP3A4 share the highest count above 50% inhibition at 10 µM. The CYP3A4 follow-up informed the switch away from the lipophilic cap variants.</t>
       </text>
     </comment>
   </commentList>
@@ -1585,7 +1585,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Reference inhibitors and historical ranges</t>
+          <t>Reference inhibitors and historical comparators</t>
         </is>
       </c>
     </row>
@@ -1755,7 +1755,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Most flagged isoform</t>
+          <t>Most flagged isoforms</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">

</xml_diff>